<commit_message>
Hogar de Refugio: tabla oficial CAPECO-FTCCP 2026 y junta longitudinal solo contra el cerco
- Hoja COSTO HORA HOMBRE 2026 con el desglose oficial CAPECO - FTCCP 2026 (Exp. 339-2025-MTPE/2.14-NC):
  28.95 / 22.68 / 20.54; todas las ACU leen de ella. PDF guardado en insumos/normas.
- 01.04.04.06.02: solo la junta longitudinal entre el muro del colector y el cimiento del cerco
  (0+000.00 a 0+058.81); al lado via hay terreno natural, sin junta: 134.89 -> 58.81 m.
  DD-03 con vista D nueva (seccion con la junta solo contra el cerco), DP-04, DP-08, DP-09, DA-03,
  especificaciones y memoria sin piso ni vereda al lado via. Se borra el esquema antiguo de juntas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/COTIZACION_PRECIOS_ACU_TAPA_REGISTRO_HOGAR_REFUGIO.xlsx
+++ b/entregables/COTIZACION_PRECIOS_ACU_TAPA_REGISTRO_HOGAR_REFUGIO.xlsx
@@ -710,7 +710,6 @@
       <c r="M3" s="34" t="n"/>
       <c r="N3" s="35" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -1981,7 +1980,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Jornal basico 2026 S/ 89.30 por dia (convenio CAPECO-FTCCP 2026, R.M. 197-2025-TR); costo hora-hombre 2026 de la hoja COSTO HORA HOMBRE 2026 de la planilla</t>
+          <t>Jornal basico 2026 S/ 89.30 por dia; costo hora-hombre en edificacion 2026 de la tabla oficial CAPECO - FTCCP (Exp. N° 339-2025-MTPE/2.14-NC)</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -1990,7 +1989,7 @@
         </is>
       </c>
       <c r="F26" s="6" t="n">
-        <v>29.3</v>
+        <v>28.95</v>
       </c>
       <c r="G26" s="18" t="n">
         <v>1</v>
@@ -2003,7 +2002,7 @@
         <v/>
       </c>
       <c r="J26" s="9" t="n">
-        <v>29.3</v>
+        <v>28.95</v>
       </c>
       <c r="K26" s="10">
         <f>I26/J26-1</f>
@@ -2011,7 +2010,7 @@
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>FTCCP - tablas salariales 2026</t>
+          <t>CAPECO - FTCCP 2026</t>
         </is>
       </c>
       <c r="M26" s="11" t="inlineStr">
@@ -2021,7 +2020,7 @@
       </c>
       <c r="N26" s="12" t="inlineStr">
         <is>
-          <t>JORNAL OFICIAL 2026; costo hh 2026 = costo CAPECO 2024-2025 x jornal 2026 / jornal 2024-2025</t>
+          <t>TABLA OFICIAL CAPECO - FTCCP 2026</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2040,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Jornal basico 2026 S/ 69.75 por dia (convenio CAPECO-FTCCP 2026, R.M. 197-2025-TR); costo hora-hombre 2026 de la hoja COSTO HORA HOMBRE 2026 de la planilla</t>
+          <t>Jornal basico 2026 S/ 69.75 por dia; costo hora-hombre en edificacion 2026 de la tabla oficial CAPECO - FTCCP (Exp. N° 339-2025-MTPE/2.14-NC)</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -2050,7 +2049,7 @@
         </is>
       </c>
       <c r="F27" s="6" t="n">
-        <v>22.95</v>
+        <v>22.68</v>
       </c>
       <c r="G27" s="18" t="n">
         <v>1</v>
@@ -2063,7 +2062,7 @@
         <v/>
       </c>
       <c r="J27" s="9" t="n">
-        <v>22.95</v>
+        <v>22.68</v>
       </c>
       <c r="K27" s="10">
         <f>I27/J27-1</f>
@@ -2071,7 +2070,7 @@
       </c>
       <c r="L27" s="5" t="inlineStr">
         <is>
-          <t>FTCCP - tablas salariales 2026</t>
+          <t>CAPECO - FTCCP 2026</t>
         </is>
       </c>
       <c r="M27" s="11" t="inlineStr">
@@ -2081,7 +2080,7 @@
       </c>
       <c r="N27" s="12" t="inlineStr">
         <is>
-          <t>JORNAL OFICIAL 2026; costo hh 2026 = costo CAPECO 2024-2025 x jornal 2026 / jornal 2024-2025</t>
+          <t>TABLA OFICIAL CAPECO - FTCCP 2026</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2100,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Jornal basico 2026 S/ 62.80 por dia (convenio CAPECO-FTCCP 2026, R.M. 197-2025-TR); costo hora-hombre 2026 de la hoja COSTO HORA HOMBRE 2026 de la planilla</t>
+          <t>Jornal basico 2026 S/ 62.80 por dia; costo hora-hombre en edificacion 2026 de la tabla oficial CAPECO - FTCCP (Exp. N° 339-2025-MTPE/2.14-NC)</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -2110,7 +2109,7 @@
         </is>
       </c>
       <c r="F28" s="6" t="n">
-        <v>20.79</v>
+        <v>20.54</v>
       </c>
       <c r="G28" s="18" t="n">
         <v>1</v>
@@ -2123,7 +2122,7 @@
         <v/>
       </c>
       <c r="J28" s="9" t="n">
-        <v>20.79</v>
+        <v>20.54</v>
       </c>
       <c r="K28" s="10">
         <f>I28/J28-1</f>
@@ -2131,7 +2130,7 @@
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>FTCCP - tablas salariales 2026</t>
+          <t>CAPECO - FTCCP 2026</t>
         </is>
       </c>
       <c r="M28" s="11" t="inlineStr">
@@ -2141,11 +2140,10 @@
       </c>
       <c r="N28" s="12" t="inlineStr">
         <is>
-          <t>JORNAL OFICIAL 2026; costo hh 2026 = costo CAPECO 2024-2025 x jornal 2026 / jornal 2024-2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="29"/>
+          <t>TABLA OFICIAL CAPECO - FTCCP 2026</t>
+        </is>
+      </c>
+    </row>
     <row r="30">
       <c r="A30" s="19" t="inlineStr">
         <is>
@@ -2269,7 +2267,7 @@
     <row r="36" ht="28" customHeight="1">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>6. Mano de obra 2026: jornal basico oficial (R.M. 197-2025-TR) y costo hora-hombre 29.30 / 22.95 / 20.79 de la hoja COSTO HORA HOMBRE 2026 de la planilla (costo CAPECO 2024-2025 llevado al jornal 2026).</t>
+          <t>6. Mano de obra 2026: costo hora-hombre 28.95 / 22.68 / 20.54 de la tabla oficial CAPECO - FTCCP 2026 (hoja COSTO HORA HOMBRE 2026 de la planilla).</t>
         </is>
       </c>
       <c r="B36" s="34" t="n"/>
@@ -2388,7 +2386,6 @@
       <c r="G3" s="34" t="n"/>
       <c r="H3" s="35" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -2611,7 +2608,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
         <is>
@@ -3087,7 +3083,6 @@
       <c r="G31" s="5" t="n"/>
       <c r="H31" s="3" t="inlineStr"/>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="19" t="inlineStr">
         <is>
@@ -3245,7 +3240,6 @@
       <c r="I3" s="34" t="n"/>
       <c r="J3" s="35" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -3457,7 +3451,6 @@
       <c r="I13" s="5" t="n"/>
       <c r="J13" s="5" t="n"/>
     </row>
-    <row r="14"/>
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>

</xml_diff>